<commit_message>
KPI actualizado 2026-07-01 20:50 UTC
</commit_message>
<xml_diff>
--- a/data/50001547 - XEMORTIZ AMERICAS GOLD.xlsx
+++ b/data/50001547 - XEMORTIZ AMERICAS GOLD.xlsx
@@ -3800,7 +3800,7 @@
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46196.70204975695</v>
+        <v>46204.860021458335</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>151</v>
@@ -3850,8 +3850,8 @@
       <c r="T40" s="6">
         <v>0</v>
       </c>
-      <c r="U40" s="12" t="s">
-        <v>103</v>
+      <c r="U40" s="11" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -3916,9 +3916,11 @@
       <c r="B42" s="5">
         <v>46156.63227357639</v>
       </c>
-      <c r="C42" s="6"/>
+      <c r="C42" s="5">
+        <v>46204.86000005787</v>
+      </c>
       <c r="D42" s="5">
-        <v>46196.699790694445</v>
+        <v>46204.86000238426</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>158</v>
@@ -3971,7 +3973,7 @@
       </c>
       <c r="C43" s="10"/>
       <c r="D43" s="9">
-        <v>46169.86151703703</v>
+        <v>46204.86001229167</v>
       </c>
       <c r="E43" s="10" t="s">
         <v>161</v>
@@ -5615,7 +5617,7 @@
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="9">
-        <v>46156.726445520835</v>
+        <v>46204.86002143519</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>248</v>
@@ -5665,8 +5667,8 @@
       <c r="T71" s="10">
         <v>0</v>
       </c>
-      <c r="U71" s="12" t="s">
-        <v>103</v>
+      <c r="U71" s="11" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-07-01 21:29 UTC
</commit_message>
<xml_diff>
--- a/data/50001547 - XEMORTIZ AMERICAS GOLD.xlsx
+++ b/data/50001547 - XEMORTIZ AMERICAS GOLD.xlsx
@@ -3798,9 +3798,11 @@
       <c r="B40" s="5">
         <v>46156.63226644676</v>
       </c>
-      <c r="C40" s="6"/>
+      <c r="C40" s="5">
+        <v>46204.87072556713</v>
+      </c>
       <c r="D40" s="5">
-        <v>46204.860021458335</v>
+        <v>46204.87074320602</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>151</v>
@@ -3848,10 +3850,10 @@
         <v>33</v>
       </c>
       <c r="T40" s="6">
-        <v>0</v>
-      </c>
-      <c r="U40" s="11" t="s">
-        <v>66</v>
+        <v>1</v>
+      </c>
+      <c r="U40" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-07-07 15:51 UTC
</commit_message>
<xml_diff>
--- a/data/50001547 - XEMORTIZ AMERICAS GOLD.xlsx
+++ b/data/50001547 - XEMORTIZ AMERICAS GOLD.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1148" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1151" uniqueCount="305">
   <si>
     <t>50001547 - XEMORTIZ (AMERICAS GOLD)</t>
   </si>
@@ -338,16 +338,16 @@
     <t>Fabricación Alabe OT 4317,Generación OC Alabe OT 4317</t>
   </si>
   <si>
+    <t>1214809660726272</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe OT 4317</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Alabe OT 4317,Alabe OT 4317 </t>
+  </si>
+  <si>
     <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1214809660726272</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe OT 4317</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Alabe OT 4317,Alabe OT 4317 </t>
   </si>
   <si>
     <t>1214809612445357</t>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46199.559805983794</v>
+        <v>46210.64699083334</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>92</v>
@@ -2740,7 +2740,9 @@
       <c r="R22" s="6"/>
       <c r="S22" s="6"/>
       <c r="T22" s="6"/>
-      <c r="U22" s="6"/>
+      <c r="U22" s="11" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
@@ -2749,9 +2751,11 @@
       <c r="B23" s="9">
         <v>46156.63213814815</v>
       </c>
-      <c r="C23" s="10"/>
+      <c r="C23" s="9">
+        <v>46210.646711388894</v>
+      </c>
       <c r="D23" s="9">
-        <v>46195.929228946756</v>
+        <v>46210.6467582176</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>95</v>
@@ -2799,15 +2803,15 @@
         <v>33</v>
       </c>
       <c r="T23" s="10">
-        <v>0</v>
-      </c>
-      <c r="U23" s="12" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="U23" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B24" s="5">
         <v>46156.63214259259</v>
@@ -2819,7 +2823,7 @@
         <v>46195.92922337963</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
@@ -2852,7 +2856,7 @@
         <v>69</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
@@ -2863,7 +2867,7 @@
         <v>0</v>
       </c>
       <c r="U24" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -2873,9 +2877,11 @@
       <c r="B25" s="9">
         <v>46156.63214717593</v>
       </c>
-      <c r="C25" s="10"/>
+      <c r="C25" s="9">
+        <v>46210.646694560186</v>
+      </c>
       <c r="D25" s="9">
-        <v>46195.92922835649</v>
+        <v>46210.64669667824</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>104</v>
@@ -2908,7 +2914,7 @@
         <v>95</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="P25" s="10" t="s">
         <v>105</v>
@@ -2922,7 +2928,7 @@
         <v>0</v>
       </c>
       <c r="U25" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
@@ -2932,9 +2938,11 @@
       <c r="B26" s="5">
         <v>46156.6321521412</v>
       </c>
-      <c r="C26" s="6"/>
+      <c r="C26" s="5">
+        <v>46210.64696896991</v>
+      </c>
       <c r="D26" s="5">
-        <v>46169.86132256944</v>
+        <v>46210.64698900463</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>107</v>
@@ -2982,10 +2990,10 @@
         <v>33</v>
       </c>
       <c r="T26" s="6">
-        <v>0</v>
-      </c>
-      <c r="U26" s="12" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="U26" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
@@ -2995,9 +3003,11 @@
       <c r="B27" s="9">
         <v>46156.63215657407</v>
       </c>
-      <c r="C27" s="10"/>
+      <c r="C27" s="9">
+        <v>46210.646919618055</v>
+      </c>
       <c r="D27" s="9">
-        <v>46197.502050625</v>
+        <v>46210.64692099537</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>110</v>
@@ -3044,7 +3054,7 @@
         <v>0</v>
       </c>
       <c r="U27" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -3054,9 +3064,11 @@
       <c r="B28" s="5">
         <v>46156.63216167824</v>
       </c>
-      <c r="C28" s="6"/>
+      <c r="C28" s="5">
+        <v>46210.64695491898</v>
+      </c>
       <c r="D28" s="5">
-        <v>46169.86172537037</v>
+        <v>46210.64695642361</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>113</v>
@@ -3103,7 +3115,7 @@
         <v>0</v>
       </c>
       <c r="U28" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -3113,9 +3125,11 @@
       <c r="B29" s="9">
         <v>46156.63216756945</v>
       </c>
-      <c r="C29" s="10"/>
+      <c r="C29" s="9">
+        <v>46210.645546747684</v>
+      </c>
       <c r="D29" s="9">
-        <v>46197.783559131945</v>
+        <v>46210.645560289355</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>116</v>
@@ -3163,10 +3177,10 @@
         <v>33</v>
       </c>
       <c r="T29" s="10">
-        <v>0</v>
-      </c>
-      <c r="U29" s="12" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="U29" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -3227,7 +3241,7 @@
         <v>0</v>
       </c>
       <c r="U30" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -3237,9 +3251,11 @@
       <c r="B31" s="9">
         <v>46156.63217837963</v>
       </c>
-      <c r="C31" s="10"/>
+      <c r="C31" s="9">
+        <v>46210.64553108797</v>
+      </c>
       <c r="D31" s="9">
-        <v>46195.92957792824</v>
+        <v>46210.64553332176</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>122</v>
@@ -3286,7 +3302,7 @@
         <v>0</v>
       </c>
       <c r="U31" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -3347,7 +3363,7 @@
         <v>0</v>
       </c>
       <c r="U32" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
@@ -3473,7 +3489,7 @@
         <v>0</v>
       </c>
       <c r="U34" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
@@ -3534,7 +3550,7 @@
         <v>0</v>
       </c>
       <c r="U35" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -3723,7 +3739,7 @@
         <v>46204.87072556713</v>
       </c>
       <c r="D39" s="9">
-        <v>46204.87074320602</v>
+        <v>46210.649648715276</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>147</v>
@@ -3894,9 +3910,11 @@
       <c r="B42" s="5">
         <v>46156.63227760416</v>
       </c>
-      <c r="C42" s="6"/>
+      <c r="C42" s="5">
+        <v>46210.649582847225</v>
+      </c>
       <c r="D42" s="5">
-        <v>46204.86001229167</v>
+        <v>46210.64958435185</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>157</v>
@@ -4417,7 +4435,7 @@
         <v>0</v>
       </c>
       <c r="U50" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
@@ -4480,9 +4498,11 @@
       <c r="B52" s="5">
         <v>46156.63233141204</v>
       </c>
-      <c r="C52" s="6"/>
+      <c r="C52" s="5">
+        <v>46210.64939368056</v>
+      </c>
       <c r="D52" s="5">
-        <v>46156.70385697916</v>
+        <v>46210.64940796296</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>194</v>
@@ -4517,8 +4537,12 @@
       <c r="Q52" s="6"/>
       <c r="R52" s="6"/>
       <c r="S52" s="6"/>
-      <c r="T52" s="6"/>
-      <c r="U52" s="6"/>
+      <c r="T52" s="6">
+        <v>1</v>
+      </c>
+      <c r="U52" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
@@ -4527,9 +4551,11 @@
       <c r="B53" s="9">
         <v>46156.63233460648</v>
       </c>
-      <c r="C53" s="10"/>
+      <c r="C53" s="9">
+        <v>46210.648792141204</v>
+      </c>
       <c r="D53" s="9">
-        <v>46199.559799317125</v>
+        <v>46210.64881278935</v>
       </c>
       <c r="E53" s="10" t="s">
         <v>197</v>
@@ -4577,10 +4603,10 @@
         <v>33</v>
       </c>
       <c r="T53" s="10">
-        <v>0</v>
-      </c>
-      <c r="U53" s="11" t="s">
-        <v>48</v>
+        <v>1</v>
+      </c>
+      <c r="U53" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
@@ -4590,9 +4616,11 @@
       <c r="B54" s="5">
         <v>46156.63233969908</v>
       </c>
-      <c r="C54" s="6"/>
+      <c r="C54" s="5">
+        <v>46210.64935451389</v>
+      </c>
       <c r="D54" s="5">
-        <v>46156.72612552083</v>
+        <v>46210.649371875</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>202</v>
@@ -4640,10 +4668,10 @@
         <v>33</v>
       </c>
       <c r="T54" s="6">
-        <v>0</v>
-      </c>
-      <c r="U54" s="12" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="U54" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
@@ -4653,9 +4681,11 @@
       <c r="B55" s="9">
         <v>46156.632350671294</v>
       </c>
-      <c r="C55" s="10"/>
+      <c r="C55" s="9">
+        <v>46210.64880347222</v>
+      </c>
       <c r="D55" s="9">
-        <v>46199.559976840275</v>
+        <v>46210.64881809028</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>206</v>
@@ -4703,10 +4733,10 @@
         <v>33</v>
       </c>
       <c r="T55" s="10">
-        <v>0</v>
-      </c>
-      <c r="U55" s="11" t="s">
-        <v>48</v>
+        <v>1</v>
+      </c>
+      <c r="U55" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
@@ -4716,9 +4746,11 @@
       <c r="B56" s="5">
         <v>46156.63235533565</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46210.64936773149</v>
+      </c>
       <c r="D56" s="5">
-        <v>46156.72612251157</v>
+        <v>46210.64938440973</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>209</v>
@@ -4766,10 +4798,10 @@
         <v>33</v>
       </c>
       <c r="T56" s="6">
-        <v>0</v>
-      </c>
-      <c r="U56" s="12" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="U56" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -4779,9 +4811,11 @@
       <c r="B57" s="9">
         <v>46156.63235945602</v>
       </c>
-      <c r="C57" s="10"/>
+      <c r="C57" s="9">
+        <v>46210.648815740744</v>
+      </c>
       <c r="D57" s="9">
-        <v>46199.56230880787</v>
+        <v>46210.648830949074</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>211</v>
@@ -4829,10 +4863,10 @@
         <v>33</v>
       </c>
       <c r="T57" s="10">
-        <v>0</v>
-      </c>
-      <c r="U57" s="11" t="s">
-        <v>48</v>
+        <v>1</v>
+      </c>
+      <c r="U57" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
@@ -4842,9 +4876,11 @@
       <c r="B58" s="5">
         <v>46156.63236322917</v>
       </c>
-      <c r="C58" s="6"/>
+      <c r="C58" s="5">
+        <v>46210.64937866898</v>
+      </c>
       <c r="D58" s="5">
-        <v>46156.72611966435</v>
+        <v>46210.64939421296</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>212</v>
@@ -4892,10 +4928,10 @@
         <v>33</v>
       </c>
       <c r="T58" s="6">
-        <v>0</v>
-      </c>
-      <c r="U58" s="12" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="U58" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -5019,7 +5055,7 @@
       </c>
       <c r="C61" s="10"/>
       <c r="D61" s="9">
-        <v>46156.72624517361</v>
+        <v>46210.64938539352</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>191</v>
@@ -5072,7 +5108,7 @@
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46205.904521226854</v>
+        <v>46210.650037060186</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>226</v>
@@ -5239,7 +5275,7 @@
         <v>0</v>
       </c>
       <c r="U64" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
@@ -5304,7 +5340,7 @@
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46156.71243400463</v>
+        <v>46210.64710428241</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>194</v>
@@ -5340,7 +5376,9 @@
       <c r="R66" s="6"/>
       <c r="S66" s="6"/>
       <c r="T66" s="6"/>
-      <c r="U66" s="6"/>
+      <c r="U66" s="11" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
@@ -5349,9 +5387,11 @@
       <c r="B67" s="9">
         <v>46156.63249635417</v>
       </c>
-      <c r="C67" s="10"/>
+      <c r="C67" s="9">
+        <v>46210.64707274306</v>
+      </c>
       <c r="D67" s="9">
-        <v>46156.72645449074</v>
+        <v>46210.64718186343</v>
       </c>
       <c r="E67" s="10" t="s">
         <v>237</v>
@@ -5399,10 +5439,10 @@
         <v>33</v>
       </c>
       <c r="T67" s="10">
-        <v>0</v>
-      </c>
-      <c r="U67" s="12" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="U67" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5412,9 +5452,11 @@
       <c r="B68" s="5">
         <v>46156.63250229167</v>
       </c>
-      <c r="C68" s="6"/>
+      <c r="C68" s="5">
+        <v>46210.647080740746</v>
+      </c>
       <c r="D68" s="5">
-        <v>46156.726451689814</v>
+        <v>46210.64712949074</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>239</v>
@@ -5462,10 +5504,10 @@
         <v>33</v>
       </c>
       <c r="T68" s="6">
-        <v>0</v>
-      </c>
-      <c r="U68" s="12" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="U68" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -5475,9 +5517,11 @@
       <c r="B69" s="9">
         <v>46156.63250851852</v>
       </c>
-      <c r="C69" s="10"/>
+      <c r="C69" s="9">
+        <v>46210.64568954861</v>
+      </c>
       <c r="D69" s="9">
-        <v>46156.726448877314</v>
+        <v>46210.645706863426</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>241</v>
@@ -5525,10 +5569,10 @@
         <v>33</v>
       </c>
       <c r="T69" s="10">
-        <v>0</v>
-      </c>
-      <c r="U69" s="12" t="s">
-        <v>99</v>
+        <v>1</v>
+      </c>
+      <c r="U69" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
@@ -5701,7 +5745,7 @@
         <v>0</v>
       </c>
       <c r="U72" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -5817,7 +5861,7 @@
         <v>0</v>
       </c>
       <c r="U74" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -5829,7 +5873,7 @@
       </c>
       <c r="C75" s="10"/>
       <c r="D75" s="9">
-        <v>46184.58084127315</v>
+        <v>46210.647096342596</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>191</v>
@@ -5933,7 +5977,7 @@
         <v>0</v>
       </c>
       <c r="U76" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -5945,7 +5989,7 @@
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="9">
-        <v>46184.58084195602</v>
+        <v>46210.64708005787</v>
       </c>
       <c r="E77" s="10" t="s">
         <v>191</v>
@@ -6049,7 +6093,7 @@
         <v>0</v>
       </c>
       <c r="U78" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
@@ -6061,7 +6105,7 @@
       </c>
       <c r="C79" s="10"/>
       <c r="D79" s="9">
-        <v>46184.58084310185</v>
+        <v>46210.645696875</v>
       </c>
       <c r="E79" s="10" t="s">
         <v>191</v>
@@ -6165,7 +6209,7 @@
         <v>0</v>
       </c>
       <c r="U80" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
@@ -6281,7 +6325,7 @@
         <v>0</v>
       </c>
       <c r="U82" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
@@ -6444,7 +6488,7 @@
         <v>0</v>
       </c>
       <c r="U85" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
@@ -6558,7 +6602,7 @@
         <v>0</v>
       </c>
       <c r="U87" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
@@ -6794,7 +6838,7 @@
         <v>0</v>
       </c>
       <c r="U91" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
@@ -6955,7 +6999,7 @@
         <v>0</v>
       </c>
       <c r="U94" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
@@ -7018,7 +7062,7 @@
         <v>0</v>
       </c>
       <c r="U95" s="12" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-09 16:49 Chile
</commit_message>
<xml_diff>
--- a/data/50001547 - XEMORTIZ AMERICAS GOLD.xlsx
+++ b/data/50001547 - XEMORTIZ AMERICAS GOLD.xlsx
@@ -2729,7 +2729,7 @@
         <v>46212.59675680556</v>
       </c>
       <c r="D22" s="5">
-        <v>46212.59677189815</v>
+        <v>46243.71324824074</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>91</v>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46156.72589140046</v>
+        <v>46243.72746450231</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>185</v>
@@ -5019,7 +5019,7 @@
         <v>46203.50147394676</v>
       </c>
       <c r="D60" s="5">
-        <v>46242.17955945602</v>
+        <v>46243.72771121528</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>217</v>
@@ -5137,7 +5137,7 @@
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46237.53857474537</v>
+        <v>46243.72774834491</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>225</v>
@@ -5253,7 +5253,7 @@
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46197.83505042824</v>
+        <v>46243.72779826389</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>230</v>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="9">
-        <v>46213.50747597222</v>
+        <v>46243.73553203704</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>245</v>
@@ -5729,7 +5729,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46237.53864697917</v>
+        <v>46243.727824525464</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>248</v>
@@ -5847,7 +5847,7 @@
         <v>46213.50741020833</v>
       </c>
       <c r="D74" s="5">
-        <v>46223.58718354166</v>
+        <v>46243.72785484954</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>252</v>
@@ -5965,7 +5965,7 @@
         <v>46213.50747125</v>
       </c>
       <c r="D76" s="5">
-        <v>46223.587179571754</v>
+        <v>46243.72789628472</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>257</v>
@@ -6081,7 +6081,7 @@
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46237.538680937505</v>
+        <v>46243.72800076389</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>261</v>
@@ -6197,7 +6197,7 @@
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46223.58716885417</v>
+        <v>46243.728052499995</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>266</v>
@@ -6313,7 +6313,7 @@
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46223.58716818287</v>
+        <v>46243.728118784726</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>270</v>
@@ -6476,7 +6476,7 @@
       </c>
       <c r="C85" s="10"/>
       <c r="D85" s="9">
-        <v>46156.7268765162</v>
+        <v>46243.72816118055</v>
       </c>
       <c r="E85" s="10" t="s">
         <v>278</v>
@@ -6592,7 +6592,7 @@
       </c>
       <c r="C87" s="10"/>
       <c r="D87" s="9">
-        <v>46223.587295798614</v>
+        <v>46243.72822305556</v>
       </c>
       <c r="E87" s="10" t="s">
         <v>284</v>
@@ -6708,7 +6708,7 @@
         <v>46205.90464569445</v>
       </c>
       <c r="D89" s="9">
-        <v>46205.904737627316</v>
+        <v>46243.72826583333</v>
       </c>
       <c r="E89" s="10" t="s">
         <v>288</v>
@@ -6826,7 +6826,7 @@
       </c>
       <c r="C91" s="10"/>
       <c r="D91" s="9">
-        <v>46156.727220243054</v>
+        <v>46243.72830107639</v>
       </c>
       <c r="E91" s="10" t="s">
         <v>292</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-20 13:52 UTC
</commit_message>
<xml_diff>
--- a/data/50001547 - XEMORTIZ AMERICAS GOLD.xlsx
+++ b/data/50001547 - XEMORTIZ AMERICAS GOLD.xlsx
@@ -5140,7 +5140,7 @@
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46243.72774834491</v>
+        <v>46254.172488854165</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>226</v>
@@ -5184,8 +5184,8 @@
       <c r="R62" s="5">
         <v>46261</v>
       </c>
-      <c r="S62" s="7" t="s">
-        <v>33</v>
+      <c r="S62" s="12" t="s">
+        <v>150</v>
       </c>
       <c r="T62" s="6">
         <v>0.5</v>

</xml_diff>